<commit_message>
Implementação de dias corridos no gráfico, inclusão de ticket e cupom na tabela
</commit_message>
<xml_diff>
--- a/Relatorio_Comissao.xlsx
+++ b/Relatorio_Comissao.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1489,38 +1489,75 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>27.632</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="H29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="I29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="J29" s="3" t="n">
-        <v>495.072</v>
-      </c>
-      <c r="K29" s="3" t="n">
-        <v>495.072</v>
+      <c r="B30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>522.704</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>522.704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>